<commit_message>
feat(data-wizard): import and export create_iam_groups on domains
</commit_message>
<xml_diff>
--- a/backend/data_wizard/import_templates/domains_template.xlsx
+++ b/backend/data_wizard/import_templates/domains_template.xlsx
@@ -404,27 +404,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
     <col width="50" customWidth="1" style="5" min="2" max="2"/>
     <col width="30" customWidth="1" style="5" min="3" max="3"/>
     <col width="30" customWidth="1" style="6" min="4" max="4"/>
+    <col width="22" customWidth="1" style="6" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" s="6">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
@@ -432,6 +433,11 @@
       <c r="D1" s="8" t="inlineStr">
         <is>
           <t>labels</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>create_iam_groups</t>
         </is>
       </c>
     </row>
@@ -441,15 +447,20 @@
           <t>ACME Corp</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Root domain for ACME</t>
         </is>
       </c>
-      <c r="C2" s="10" t="n"/>
+      <c r="C2" s="11" t="n"/>
       <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Group</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -459,12 +470,12 @@
           <t>IT Department</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>All IT assets and</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>ACME Corp</t>
         </is>
@@ -472,6 +483,11 @@
       <c r="D3" s="11" t="inlineStr">
         <is>
           <t>IT</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -481,12 +497,12 @@
           <t>HR Department</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Human Resources scope</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>ACME Corp</t>
         </is>
@@ -494,6 +510,11 @@
       <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Corporate</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -503,12 +524,12 @@
           <t>Finance</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Financial systems and data</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>ACME Corp</t>
         </is>
@@ -516,6 +537,11 @@
       <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Corporate,Finance</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -532,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="5" min="1" max="1"/>
@@ -541,70 +567,70 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="6">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2" ht="45" customHeight="1" s="6">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Unique name for the folder/domain. Used for conflict detection together with 'domain'.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="45" customHeight="1" s="6">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Free-text description of the folder.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1" s="6">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Name of the parent folder. Leave blank to place the folder at root level. Must match exactly one existing folder name (case-insensitive). An error is returned when the name is ambiguous.</t>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Name of the parent domain. Leave blank to place the folder at root level. Must match exactly one existing domain name (case-insensitive), unless the row's internal_id points to a domain whose current parent has that name.</t>
         </is>
       </c>
     </row>
@@ -621,7 +647,24 @@
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Filtering labels attached to the folder, separated by commas or pipes (e.g. "Corporate,Finance"). Labels that do not exist yet are created. Also accepted as column "label" or "filtering_labels".</t>
+          <t>Filtering labels attached to the folder, separated by commas or pipes (e.g. "Corporate,Finance"). Labels that do not exist yet are created, which requires the permission to add labels. Also accepted as column "label" or "filtering_labels".</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>create_iam_groups</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Whether the domain gets its IAM groups (true/false, yes/no or 1/0). Blank keeps the default (false) on creation and leaves an existing domain untouched.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(folders): add ref_id, unique per parent folder
</commit_message>
<xml_diff>
--- a/backend/data_wizard/import_templates/domains_template.xlsx
+++ b/backend/data_wizard/import_templates/domains_template.xlsx
@@ -404,38 +404,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="30" customWidth="1" style="5" min="1" max="1"/>
-    <col width="50" customWidth="1" style="5" min="2" max="2"/>
-    <col width="30" customWidth="1" style="5" min="3" max="3"/>
-    <col width="30" customWidth="1" style="6" min="4" max="4"/>
-    <col width="22" customWidth="1" style="6" min="5" max="5"/>
+    <col width="15" customWidth="1" style="5" min="1" max="1"/>
+    <col width="30" customWidth="1" style="5" min="2" max="2"/>
+    <col width="50" customWidth="1" style="5" min="3" max="3"/>
+    <col width="30" customWidth="1" style="5" min="4" max="4"/>
+    <col width="30" customWidth="1" style="6" min="5" max="5"/>
+    <col width="22" customWidth="1" style="6" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" s="6">
       <c r="A1" s="8" t="inlineStr">
         <is>
+          <t>ref_id</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>labels</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>create_iam_groups</t>
         </is>
@@ -444,21 +450,26 @@
     <row r="2" ht="18" customHeight="1" s="6">
       <c r="A2" s="9" t="inlineStr">
         <is>
+          <t>DOM.01</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
           <t>ACME Corp</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Root domain for ACME</t>
         </is>
       </c>
-      <c r="C2" s="11" t="n"/>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="11" t="n"/>
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -467,25 +478,30 @@
     <row r="3" ht="18" customHeight="1" s="6">
       <c r="A3" s="9" t="inlineStr">
         <is>
+          <t>DOM.IT</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
           <t>IT Department</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>All IT assets and</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>ACME Corp</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -494,25 +510,30 @@
     <row r="4" ht="18" customHeight="1" s="6">
       <c r="A4" s="9" t="inlineStr">
         <is>
+          <t>DOM.HR</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
           <t>HR Department</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Human Resources scope</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>ACME Corp</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Corporate</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -521,25 +542,30 @@
     <row r="5" ht="18" customHeight="1" s="6">
       <c r="A5" s="9" t="inlineStr">
         <is>
+          <t>DOM.FIN</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Financial systems and data</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>ACME Corp</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Corporate,Finance</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -558,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="5" min="1" max="1"/>
@@ -586,41 +612,41 @@
     <row r="2" ht="45" customHeight="1" s="6">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>ref_id</t>
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>Unique name for the folder/domain. Used for conflict detection together with 'domain'.</t>
+          <t>Reference ID of the folder (free text).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="45" customHeight="1" s="6">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Free-text description of the folder.</t>
+          <t>Unique name for the folder/domain. Used for conflict detection together with 'domain'.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1" s="6">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>domain</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
@@ -630,14 +656,14 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>Name of the parent domain. Leave blank to place the folder at root level. Must match exactly one existing domain name (case-insensitive), unless the row's internal_id points to a domain whose current parent has that name.</t>
+          <t>Free-text description of the folder.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>labels</t>
+          <t>domain</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
@@ -647,22 +673,39 @@
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Filtering labels attached to the folder, separated by commas or pipes (e.g. "Corporate,Finance"). Labels that do not exist yet are created, which requires the permission to add labels. Also accepted as column "label" or "filtering_labels".</t>
+          <t>Name of the parent domain. Leave blank to place the folder at root level. Must match exactly one existing domain name (case-insensitive), unless the row's internal_id points to a domain whose current parent has that name.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
+          <t>labels</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Filtering labels attached to the folder, separated by commas or pipes (e.g. "Corporate,Finance"). Labels that do not exist yet are created, which requires the permission to add labels. Also accepted as column "label" or "filtering_labels".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
           <t>create_iam_groups</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>Whether the domain gets its IAM groups (true/false, yes/no or 1/0). Blank keeps the default (false) on creation and leaves an existing domain untouched.</t>
         </is>

</xml_diff>

<commit_message>
feat(folders): add ref_id, unique across all folders (#5077)
* feat(folders): add ref_id, unique per parent folder

* fix(folders): treat whitespace-only ref_id as blank

* fix(folders): index the trimmed ref_id

* feat(folders): make ref_id unique across all folders

* fix(search): search folders by ref_id

* fix(folders): trim ref_id whitespace alike in clean() and index, map constraint race to 400

* refactor(folders): one ref_id duplicate check, report name and ref_id clashes together

---------

Co-authored-by: Abder <smimite@gmail.com>
</commit_message>
<xml_diff>
--- a/backend/data_wizard/import_templates/domains_template.xlsx
+++ b/backend/data_wizard/import_templates/domains_template.xlsx
@@ -404,38 +404,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="30" customWidth="1" style="5" min="1" max="1"/>
-    <col width="50" customWidth="1" style="5" min="2" max="2"/>
-    <col width="30" customWidth="1" style="5" min="3" max="3"/>
-    <col width="30" customWidth="1" style="6" min="4" max="4"/>
-    <col width="22" customWidth="1" style="6" min="5" max="5"/>
+    <col width="15" customWidth="1" style="5" min="1" max="1"/>
+    <col width="30" customWidth="1" style="5" min="2" max="2"/>
+    <col width="50" customWidth="1" style="5" min="3" max="3"/>
+    <col width="30" customWidth="1" style="5" min="4" max="4"/>
+    <col width="30" customWidth="1" style="6" min="5" max="5"/>
+    <col width="22" customWidth="1" style="6" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" s="6">
       <c r="A1" s="8" t="inlineStr">
         <is>
+          <t>ref_id</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>labels</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>create_iam_groups</t>
         </is>
@@ -444,21 +450,26 @@
     <row r="2" ht="18" customHeight="1" s="6">
       <c r="A2" s="9" t="inlineStr">
         <is>
+          <t>DOM.01</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
           <t>ACME Corp</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Root domain for ACME</t>
         </is>
       </c>
-      <c r="C2" s="11" t="n"/>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="11" t="n"/>
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -467,25 +478,30 @@
     <row r="3" ht="18" customHeight="1" s="6">
       <c r="A3" s="9" t="inlineStr">
         <is>
+          <t>DOM.IT</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
           <t>IT Department</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>All IT assets and</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>ACME Corp</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -494,25 +510,30 @@
     <row r="4" ht="18" customHeight="1" s="6">
       <c r="A4" s="9" t="inlineStr">
         <is>
+          <t>DOM.HR</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
           <t>HR Department</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Human Resources scope</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>ACME Corp</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Corporate</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -521,25 +542,30 @@
     <row r="5" ht="18" customHeight="1" s="6">
       <c r="A5" s="9" t="inlineStr">
         <is>
+          <t>DOM.FIN</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Financial systems and data</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>ACME Corp</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Corporate,Finance</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -558,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="5" min="1" max="1"/>
@@ -586,41 +612,41 @@
     <row r="2" ht="45" customHeight="1" s="6">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>ref_id</t>
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>Unique name for the folder/domain. Used for conflict detection together with 'domain'.</t>
+          <t>Reference ID of the folder (free text).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="45" customHeight="1" s="6">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Free-text description of the folder.</t>
+          <t>Unique name for the folder/domain. Used for conflict detection together with 'domain'.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1" s="6">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>domain</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
@@ -630,14 +656,14 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>Name of the parent domain. Leave blank to place the folder at root level. Must match exactly one existing domain name (case-insensitive), unless the row's internal_id points to a domain whose current parent has that name.</t>
+          <t>Free-text description of the folder.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>labels</t>
+          <t>domain</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
@@ -647,22 +673,39 @@
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Filtering labels attached to the folder, separated by commas or pipes (e.g. "Corporate,Finance"). Labels that do not exist yet are created, which requires the permission to add labels. Also accepted as column "label" or "filtering_labels".</t>
+          <t>Name of the parent domain. Leave blank to place the folder at root level. Must match exactly one existing domain name (case-insensitive), unless the row's internal_id points to a domain whose current parent has that name.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
+          <t>labels</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Filtering labels attached to the folder, separated by commas or pipes (e.g. "Corporate,Finance"). Labels that do not exist yet are created, which requires the permission to add labels. Also accepted as column "label" or "filtering_labels".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
           <t>create_iam_groups</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>Whether the domain gets its IAM groups (true/false, yes/no or 1/0). Blank keeps the default (false) on creation and leaves an existing domain untouched.</t>
         </is>

</xml_diff>